<commit_message>
Admin: update Genshin Impact leaks
</commit_message>
<xml_diff>
--- a/banners/02_Genshin_Impact_leaks.xlsx
+++ b/banners/02_Genshin_Impact_leaks.xlsx
@@ -65,28 +65,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7.2</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-06</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-27</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.16, 2.8, 2.22</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>